<commit_message>
docs(j4): mise a jour des documents de gestion apres sprint 5, documents liés à la perturbation j4 et mise a jour des plans sprint 6 et 7 pour s'adapter aux nouvelles US amenées par la perturbation j4
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-sprint-backlog-v5.0.xlsx
+++ b/docs/cadrage/equipe-09-sprint-backlog-v5.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="14"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" state="visible" r:id="rId3"/>
@@ -20,7 +20,11 @@
     <sheet name="Burndown Sprint 4" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Sprint 5" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="Burndown Sprint 5" sheetId="12" state="visible" r:id="rId14"/>
-    <sheet name="Auto-évaluation" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="Sprint 6" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="Burndown Sprint 6" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="Sprint 7" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Burndown Sprint 7" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="Auto-évaluation" sheetId="17" state="visible" r:id="rId19"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -32,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="328">
   <si>
     <t xml:space="preserve">A</t>
   </si>
@@ -73,19 +77,19 @@
     <t xml:space="preserve">Sprint concerné</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 5</t>
+    <t xml:space="preserve">Sprint 7</t>
   </si>
   <si>
     <t xml:space="preserve">Version</t>
   </si>
   <si>
-    <t xml:space="preserve">V5.0</t>
+    <t xml:space="preserve">V7.0</t>
   </si>
   <si>
     <t xml:space="preserve">Date de remise</t>
   </si>
   <si>
-    <t xml:space="preserve">01/07/2026 18h00</t>
+    <t xml:space="preserve">02/07/2026 18h00</t>
   </si>
   <si>
     <t xml:space="preserve">Statut</t>
@@ -639,7 +643,7 @@
     <t xml:space="preserve">Sprint 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Mercredi 31/07/2026, 9h00 à 13h00 (4 h)</t>
+    <t xml:space="preserve">Mercredi 01/07/2026, 9h00 à 13h00 (4 h)</t>
   </si>
   <si>
     <t xml:space="preserve">sécurisation prompt injection (perturbation J3)+ Conformité RGPD SAR (J3-bis) 
@@ -733,7 +737,10 @@
     <t xml:space="preserve">SPRINT BACKLOG : SPRINT 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Mercredi 31/07/2026, 13h00 à 18h00 (4 h)</t>
+    <t xml:space="preserve">Sprint 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercredi 01/07/2026, 13h00 à 18h00 (4 h)</t>
   </si>
   <si>
     <t xml:space="preserve">Difficulté + historique</t>
@@ -748,67 +755,209 @@
     <t xml:space="preserve">Endpoint GET /api/courses/ — liste paginée filtrée request.user</t>
   </si>
   <si>
+    <t xml:space="preserve">T-08.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serializer + annotate nb_quizz + tests API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page frontend /library + empty state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route /library + lien nav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests pytest anti-fuite + vitest LibraryPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST /api/quizzes/generate/ — difficulty + nb_questions (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patch quiz_prompt.py — 3 niveaux + nb variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI difficulté + slider 5-20 sur GenerateQuizPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests pytest génération (bornes + niveaux)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note doc critères CA US-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BURNDOWN : SPRINT 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPRINT BACKLOG : SPRINT 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeudi 01/07/2026, 9h00 à 13h00 (4 h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 personnes (absence Ryma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 × 4 h = 16 h-pers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 SP (US-25 = 5 · US-26 = 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accessibilité RGAA parcours F1–F6 (US-25) + i18n interface FR/EN/ES (US-26)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-25.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audit Lighthouse + axe DevTools sur /login /signup /upload /quiz /resultat — rapport 10 écarts P1 RGAA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Todo</t>
   </si>
   <si>
-    <t xml:space="preserve">T-08.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serializer + annotate nb_quizz + tests API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-08.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page frontend /library + empty state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-08.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Route /library + lien nav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-08.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tests pytest anti-fuite + vitest LibraryPage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-09.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POST /api/quizzes/generate/ — difficulty + nb_questions (5-20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-09.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patch quiz_prompt.py — 3 niveaux + nb variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-09.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI difficulté + slider 5-20 sur GenerateQuizPage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-09.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tests pytest génération (bornes + niveaux)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-09.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note doc critères CA US-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BURNDOWN : SPRINT 5</t>
+    <t xml:space="preserve">T-25.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSS focus-visible + contrastes ≥ 4,5:1 (index.css + composants Button/Input)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-25.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARIA + sémantique (header/main/nav/label) — LoginPage, SignupPage, UploadPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-25.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QuizPage : navigation clavier (radios, Tab, Enter pour soumettre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-26.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">npm react-i18next + I18nextProvider main.tsx + locales/fr.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-26.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Externaliser textes FR — Login, Signup, Upload, Quiz, Result, History</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-26.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">locales/en.json + locales/es.json (mêmes pages) + fallback FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-26.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composant LanguageSwitcher header + persistance localStorage i18n_lang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BURNDOWN : SPRINT 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPRINT BACKLOG : SPRINT 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeudi 02/07/2026, 13h00 à 18h00 (4 h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docker-compose.native.yml — image Ollama 8B+ GPU (gpus: all) + .env.prod.example (LLM_MODEL, OLLAMA_HOST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">settings.py — OLLAMA_NUM_CTX / NUM_PREDICT / timeout workers pour cours 8k+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ollama_client.py — retries JSON + feedback prompt + tests pytest 10 générations cours 8k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test de charge k6 (100 VUs) génération quiz + rapport archivé docs/sprint-7/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runbook déploiement LLM 8B (pull model, healthcheck, rollback) + make dev-native</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest perf — p95 &lt; 30 s et taux échec JSON &lt; 10 % sur 20 essais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpoint ou script healthcheck LLM + smoke test CI (mock si GPU indispo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-27.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revue ADR scalabilité + alignement équipe + vérif critères CA US-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BURNDOWN : SPRINT 7</t>
   </si>
   <si>
     <t xml:space="preserve">✅ Grille d'auto-évaluation</t>
@@ -884,7 +1033,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1114,12 +1263,6 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF1E1B4B"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
   </fonts>
   <fills count="16">
     <fill>
@@ -1277,7 +1420,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1494,15 +1637,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2049,7 +2188,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>13</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2057,7 +2196,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2088,8 +2227,8 @@
       <c r="A10" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="54" t="s">
-        <v>233</v>
+      <c r="B10" s="51" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2164,233 +2303,233 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="55" t="s">
-        <v>234</v>
-      </c>
-      <c r="B20" s="55" t="s">
+      <c r="A20" s="54" t="s">
         <v>235</v>
       </c>
-      <c r="C20" s="55" t="s">
+      <c r="B20" s="54" t="s">
         <v>236</v>
       </c>
-      <c r="D20" s="55" t="s">
+      <c r="C20" s="54" t="s">
+        <v>237</v>
+      </c>
+      <c r="D20" s="54" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="55" t="n">
+      <c r="E20" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="55" t="n">
+      <c r="F20" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="55" t="s">
-        <v>237</v>
+      <c r="G20" s="54" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="55" t="s">
-        <v>234</v>
-      </c>
-      <c r="B21" s="55" t="s">
+      <c r="A21" s="54" t="s">
+        <v>235</v>
+      </c>
+      <c r="B21" s="54" t="s">
         <v>238</v>
       </c>
-      <c r="C21" s="55" t="s">
+      <c r="C21" s="54" t="s">
         <v>239</v>
       </c>
-      <c r="D21" s="55" t="s">
+      <c r="D21" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="55" t="n">
+      <c r="E21" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="55" t="n">
+      <c r="F21" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="55" t="s">
-        <v>237</v>
+      <c r="G21" s="54" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="55" t="s">
-        <v>234</v>
-      </c>
-      <c r="B22" s="55" t="s">
+      <c r="A22" s="54" t="s">
+        <v>235</v>
+      </c>
+      <c r="B22" s="54" t="s">
         <v>240</v>
       </c>
-      <c r="C22" s="55" t="s">
+      <c r="C22" s="54" t="s">
         <v>241</v>
       </c>
-      <c r="D22" s="55" t="s">
+      <c r="D22" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="55" t="n">
+      <c r="E22" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="55" t="n">
+      <c r="F22" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="55" t="s">
-        <v>237</v>
+      <c r="G22" s="54" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="55" t="s">
-        <v>234</v>
-      </c>
-      <c r="B23" s="55" t="s">
+      <c r="A23" s="54" t="s">
+        <v>235</v>
+      </c>
+      <c r="B23" s="54" t="s">
         <v>242</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="54" t="s">
         <v>243</v>
       </c>
-      <c r="D23" s="55" t="s">
+      <c r="D23" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="E23" s="55" t="n">
+      <c r="E23" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="55" t="n">
+      <c r="F23" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="55" t="s">
-        <v>237</v>
+      <c r="G23" s="54" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="42.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="55" t="s">
-        <v>234</v>
-      </c>
-      <c r="B24" s="55" t="s">
+      <c r="A24" s="54" t="s">
+        <v>235</v>
+      </c>
+      <c r="B24" s="54" t="s">
         <v>244</v>
       </c>
-      <c r="C24" s="55" t="s">
+      <c r="C24" s="54" t="s">
         <v>245</v>
       </c>
-      <c r="D24" s="55" t="s">
+      <c r="D24" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="E24" s="55" t="n">
+      <c r="E24" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="55" t="n">
+      <c r="F24" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="55" t="s">
-        <v>237</v>
+      <c r="G24" s="54" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="40.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="56" t="s">
+      <c r="A25" s="55" t="s">
         <v>246</v>
       </c>
-      <c r="B25" s="56" t="s">
+      <c r="B25" s="55" t="s">
         <v>247</v>
       </c>
-      <c r="C25" s="56" t="s">
+      <c r="C25" s="55" t="s">
         <v>248</v>
       </c>
-      <c r="D25" s="56" t="s">
+      <c r="D25" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="E25" s="56" t="n">
+      <c r="E25" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="56" t="n">
+      <c r="F25" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="56" t="s">
-        <v>237</v>
+      <c r="G25" s="55" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="41.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="56" t="s">
+      <c r="A26" s="55" t="s">
         <v>246</v>
       </c>
-      <c r="B26" s="56" t="s">
+      <c r="B26" s="55" t="s">
         <v>249</v>
       </c>
-      <c r="C26" s="56" t="s">
+      <c r="C26" s="55" t="s">
         <v>250</v>
       </c>
-      <c r="D26" s="56" t="s">
+      <c r="D26" s="55" t="s">
         <v>78</v>
       </c>
-      <c r="E26" s="56" t="n">
+      <c r="E26" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="56" t="n">
+      <c r="F26" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="56" t="s">
-        <v>237</v>
+      <c r="G26" s="55" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="56" t="s">
+      <c r="A27" s="55" t="s">
         <v>246</v>
       </c>
-      <c r="B27" s="56" t="s">
+      <c r="B27" s="55" t="s">
         <v>251</v>
       </c>
-      <c r="C27" s="56" t="s">
+      <c r="C27" s="55" t="s">
         <v>252</v>
       </c>
-      <c r="D27" s="56" t="s">
+      <c r="D27" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="E27" s="56" t="n">
+      <c r="E27" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="56" t="n">
+      <c r="F27" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="56" t="s">
-        <v>237</v>
+      <c r="G27" s="55" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="56" t="s">
+      <c r="A28" s="55" t="s">
         <v>246</v>
       </c>
-      <c r="B28" s="56" t="s">
+      <c r="B28" s="55" t="s">
         <v>253</v>
       </c>
-      <c r="C28" s="56" t="s">
+      <c r="C28" s="55" t="s">
         <v>254</v>
       </c>
-      <c r="D28" s="56" t="s">
+      <c r="D28" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="E28" s="56" t="n">
+      <c r="E28" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="F28" s="56" t="n">
+      <c r="F28" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="56" t="s">
-        <v>237</v>
+      <c r="G28" s="55" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="56" t="s">
+      <c r="A29" s="55" t="s">
         <v>246</v>
       </c>
-      <c r="B29" s="56" t="s">
+      <c r="B29" s="55" t="s">
         <v>255</v>
       </c>
-      <c r="C29" s="56" t="s">
+      <c r="C29" s="55" t="s">
         <v>256</v>
       </c>
-      <c r="D29" s="56" t="s">
+      <c r="D29" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="E29" s="56" t="n">
+      <c r="E29" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="56" t="n">
+      <c r="F29" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="56" t="s">
-        <v>237</v>
+      <c r="G29" s="55" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2523,8 +2662,12 @@
       <c r="B8" s="39" t="n">
         <v>13</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
+      <c r="C8" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="E8" s="19" t="s">
         <v>102</v>
       </c>
@@ -2536,8 +2679,12 @@
       <c r="B9" s="39" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
+      <c r="C9" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="39" t="n">
+        <v>2</v>
+      </c>
       <c r="E9" s="19" t="s">
         <v>104</v>
       </c>
@@ -2549,8 +2696,12 @@
       <c r="B10" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
+      <c r="C10" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="39" t="n">
+        <v>5</v>
+      </c>
       <c r="E10" s="19" t="s">
         <v>106</v>
       </c>
@@ -2562,8 +2713,12 @@
       <c r="B11" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
+      <c r="C11" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="39" t="n">
+        <v>4</v>
+      </c>
       <c r="E11" s="19" t="s">
         <v>108</v>
       </c>
@@ -2575,8 +2730,12 @@
       <c r="B12" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
+      <c r="C12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="E12" s="19" t="s">
         <v>110</v>
       </c>
@@ -2642,6 +2801,1162 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="51" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="32.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B20" s="52" t="s">
+        <v>266</v>
+      </c>
+      <c r="C20" s="52" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="52" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B21" s="52" t="s">
+        <v>269</v>
+      </c>
+      <c r="C21" s="52" t="s">
+        <v>270</v>
+      </c>
+      <c r="D21" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="52" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B22" s="52" t="s">
+        <v>271</v>
+      </c>
+      <c r="C22" s="52" t="s">
+        <v>272</v>
+      </c>
+      <c r="D22" s="52" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="52" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="42.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="52" t="s">
+        <v>265</v>
+      </c>
+      <c r="B23" s="52" t="s">
+        <v>273</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>274</v>
+      </c>
+      <c r="D23" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="52" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="40.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="B24" s="53" t="s">
+        <v>276</v>
+      </c>
+      <c r="C24" s="53" t="s">
+        <v>277</v>
+      </c>
+      <c r="D24" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="53" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="41.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="B25" s="53" t="s">
+        <v>278</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>279</v>
+      </c>
+      <c r="D25" s="53" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="53" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="B26" s="53" t="s">
+        <v>280</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>281</v>
+      </c>
+      <c r="D26" s="53" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="53" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="B27" s="53" t="s">
+        <v>282</v>
+      </c>
+      <c r="C27" s="53" t="s">
+        <v>283</v>
+      </c>
+      <c r="D27" s="53" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="53" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="34"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="F28" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="G28" s="34"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1048570" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="35"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="38" t="s">
+        <v>226</v>
+      </c>
+      <c r="B8" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="B10" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="38" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="38" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="51" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="54" t="s">
+        <v>288</v>
+      </c>
+      <c r="B20" s="54" t="s">
+        <v>289</v>
+      </c>
+      <c r="C20" s="54" t="s">
+        <v>290</v>
+      </c>
+      <c r="D20" s="54" t="s">
+        <v>73</v>
+      </c>
+      <c r="E20" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="54" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="54" t="s">
+        <v>288</v>
+      </c>
+      <c r="B21" s="54" t="s">
+        <v>291</v>
+      </c>
+      <c r="C21" s="54" t="s">
+        <v>292</v>
+      </c>
+      <c r="D21" s="54" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="54" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="54" t="s">
+        <v>288</v>
+      </c>
+      <c r="B22" s="54" t="s">
+        <v>293</v>
+      </c>
+      <c r="C22" s="54" t="s">
+        <v>294</v>
+      </c>
+      <c r="D22" s="54" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="54" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="42.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="54" t="s">
+        <v>288</v>
+      </c>
+      <c r="B23" s="54" t="s">
+        <v>295</v>
+      </c>
+      <c r="C23" s="54" t="s">
+        <v>296</v>
+      </c>
+      <c r="D23" s="54" t="s">
+        <v>141</v>
+      </c>
+      <c r="E23" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="54" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="40.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="55" t="s">
+        <v>288</v>
+      </c>
+      <c r="B24" s="55" t="s">
+        <v>297</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>298</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>141</v>
+      </c>
+      <c r="E24" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="55" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="41.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="55" t="s">
+        <v>288</v>
+      </c>
+      <c r="B25" s="55" t="s">
+        <v>299</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>300</v>
+      </c>
+      <c r="D25" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="55" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="55" t="s">
+        <v>288</v>
+      </c>
+      <c r="B26" s="55" t="s">
+        <v>301</v>
+      </c>
+      <c r="C26" s="55" t="s">
+        <v>302</v>
+      </c>
+      <c r="D26" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="55" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="55" t="s">
+        <v>288</v>
+      </c>
+      <c r="B27" s="55" t="s">
+        <v>303</v>
+      </c>
+      <c r="C27" s="55" t="s">
+        <v>304</v>
+      </c>
+      <c r="D27" s="55" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="55" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="34"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="F28" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="G28" s="34"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1048570" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="35"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A2:D15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2653,126 +3968,126 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>258</v>
+        <v>306</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
-        <v>259</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23"/>
       <c r="B5" s="23" t="s">
-        <v>260</v>
+        <v>308</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>261</v>
+        <v>309</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>262</v>
+        <v>310</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="57" t="s">
-        <v>263</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D6" s="57" t="s">
-        <v>265</v>
+      <c r="B6" s="56" t="s">
+        <v>311</v>
+      </c>
+      <c r="C6" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D6" s="56" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="57" t="s">
-        <v>266</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D7" s="57" t="s">
-        <v>267</v>
+      <c r="B7" s="56" t="s">
+        <v>314</v>
+      </c>
+      <c r="C7" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D7" s="56" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="57" t="s">
-        <v>268</v>
-      </c>
-      <c r="C8" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D8" s="57" t="s">
-        <v>269</v>
+      <c r="B8" s="56" t="s">
+        <v>316</v>
+      </c>
+      <c r="C8" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D8" s="56" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="57" t="s">
-        <v>270</v>
-      </c>
-      <c r="C9" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D9" s="57" t="s">
-        <v>271</v>
+      <c r="B9" s="56" t="s">
+        <v>318</v>
+      </c>
+      <c r="C9" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D9" s="56" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="57" t="s">
-        <v>272</v>
-      </c>
-      <c r="C10" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D10" s="57"/>
+      <c r="B10" s="56" t="s">
+        <v>320</v>
+      </c>
+      <c r="C10" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D10" s="56"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="57" t="s">
-        <v>273</v>
-      </c>
-      <c r="C11" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D11" s="57" t="s">
-        <v>274</v>
+      <c r="B11" s="56" t="s">
+        <v>321</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D11" s="56" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="57" t="s">
-        <v>275</v>
-      </c>
-      <c r="C12" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D12" s="57"/>
+      <c r="B12" s="56" t="s">
+        <v>323</v>
+      </c>
+      <c r="C12" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D12" s="56"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="57" t="s">
-        <v>276</v>
-      </c>
-      <c r="C13" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D13" s="57"/>
+      <c r="B13" s="56" t="s">
+        <v>324</v>
+      </c>
+      <c r="C13" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D13" s="56"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="57" t="s">
-        <v>277</v>
-      </c>
-      <c r="C14" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D14" s="57"/>
+      <c r="B14" s="56" t="s">
+        <v>325</v>
+      </c>
+      <c r="C14" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D14" s="56"/>
     </row>
     <row r="15" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="57" t="s">
-        <v>278</v>
-      </c>
-      <c r="C15" s="58" t="s">
-        <v>264</v>
-      </c>
-      <c r="D15" s="57" t="s">
-        <v>279</v>
+      <c r="B15" s="56" t="s">
+        <v>326</v>
+      </c>
+      <c r="C15" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="D15" s="56" t="s">
+        <v>327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>